<commit_message>
Termine de modificar formatos de la base construida
</commit_message>
<xml_diff>
--- a/Datos/Procesados/base_construida.xlsx
+++ b/Datos/Procesados/base_construida.xlsx
@@ -15,6 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -52,11 +55,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -353,6 +357,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB127"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
@@ -497,8 +504,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>16709</v>
+      <c r="A2" s="2">
+        <v>42278</v>
       </c>
       <c r="E2">
         <v>116</v>
@@ -575,8 +582,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>16740</v>
+      <c r="A3" s="2">
+        <v>42309</v>
       </c>
       <c r="E3">
         <v>97</v>
@@ -653,8 +660,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>16770</v>
+      <c r="A4" s="2">
+        <v>42339</v>
       </c>
       <c r="E4">
         <v>107</v>
@@ -731,8 +738,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <v>16801</v>
+      <c r="A5" s="2">
+        <v>42370</v>
       </c>
       <c r="E5">
         <v>98</v>
@@ -809,8 +816,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <v>16832</v>
+      <c r="A6" s="2">
+        <v>42401</v>
       </c>
       <c r="E6">
         <v>96</v>
@@ -887,8 +894,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <v>16861</v>
+      <c r="A7" s="2">
+        <v>42430</v>
       </c>
       <c r="E7">
         <v>85</v>
@@ -965,8 +972,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <v>16892</v>
+      <c r="A8" s="2">
+        <v>42461</v>
       </c>
       <c r="E8">
         <v>106</v>
@@ -1043,8 +1050,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9">
-        <v>16922</v>
+      <c r="A9" s="2">
+        <v>42491</v>
       </c>
       <c r="E9">
         <v>97</v>
@@ -1121,8 +1128,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10">
-        <v>16953</v>
+      <c r="A10" s="2">
+        <v>42522</v>
       </c>
       <c r="E10">
         <v>104</v>
@@ -1199,8 +1206,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11">
-        <v>16983</v>
+      <c r="A11" s="2">
+        <v>42552</v>
       </c>
       <c r="E11">
         <v>112</v>
@@ -1277,8 +1284,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12">
-        <v>17014</v>
+      <c r="A12" s="2">
+        <v>42583</v>
       </c>
       <c r="E12">
         <v>95</v>
@@ -1355,8 +1362,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <v>17045</v>
+      <c r="A13" s="2">
+        <v>42614</v>
       </c>
       <c r="E13">
         <v>101</v>
@@ -1433,8 +1440,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <v>17075</v>
+      <c r="A14" s="2">
+        <v>42644</v>
       </c>
       <c r="E14">
         <v>92</v>
@@ -1511,8 +1518,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15">
-        <v>17106</v>
+      <c r="A15" s="2">
+        <v>42675</v>
       </c>
       <c r="E15">
         <v>116</v>
@@ -1589,8 +1596,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <v>17136</v>
+      <c r="A16" s="2">
+        <v>42705</v>
       </c>
       <c r="E16">
         <v>132</v>
@@ -1667,8 +1674,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17">
-        <v>17167</v>
+      <c r="A17" s="2">
+        <v>42736</v>
       </c>
       <c r="E17">
         <v>153</v>
@@ -1745,8 +1752,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18">
-        <v>17198</v>
+      <c r="A18" s="2">
+        <v>42767</v>
       </c>
       <c r="E18">
         <v>134</v>
@@ -1823,8 +1830,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19">
-        <v>17226</v>
+      <c r="A19" s="2">
+        <v>42795</v>
       </c>
       <c r="E19">
         <v>124</v>
@@ -1901,8 +1908,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20">
-        <v>17257</v>
+      <c r="A20" s="2">
+        <v>42826</v>
       </c>
       <c r="E20">
         <v>130</v>
@@ -1979,8 +1986,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21">
-        <v>17287</v>
+      <c r="A21" s="2">
+        <v>42856</v>
       </c>
       <c r="E21">
         <v>130</v>
@@ -2057,8 +2064,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22">
-        <v>17318</v>
+      <c r="A22" s="2">
+        <v>42887</v>
       </c>
       <c r="E22">
         <v>131</v>
@@ -2135,8 +2142,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23">
-        <v>17348</v>
+      <c r="A23" s="2">
+        <v>42917</v>
       </c>
       <c r="E23">
         <v>139</v>
@@ -2213,8 +2220,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24">
-        <v>17379</v>
+      <c r="A24" s="2">
+        <v>42948</v>
       </c>
       <c r="E24">
         <v>132</v>
@@ -2291,8 +2298,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25">
-        <v>17410</v>
+      <c r="A25" s="2">
+        <v>42979</v>
       </c>
       <c r="E25">
         <v>132</v>
@@ -2369,8 +2376,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26">
-        <v>17440</v>
+      <c r="A26" s="2">
+        <v>43009</v>
       </c>
       <c r="E26">
         <v>135</v>
@@ -2447,8 +2454,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27">
-        <v>17471</v>
+      <c r="A27" s="2">
+        <v>43040</v>
       </c>
       <c r="E27">
         <v>128</v>
@@ -2525,8 +2532,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28">
-        <v>17501</v>
+      <c r="A28" s="2">
+        <v>43070</v>
       </c>
       <c r="E28">
         <v>126</v>
@@ -2603,8 +2610,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29">
-        <v>17532</v>
+      <c r="A29" s="2">
+        <v>43101</v>
       </c>
       <c r="E29">
         <v>135</v>
@@ -2681,8 +2688,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30">
-        <v>17563</v>
+      <c r="A30" s="2">
+        <v>43132</v>
       </c>
       <c r="E30">
         <v>140</v>
@@ -2759,8 +2766,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31">
-        <v>17591</v>
+      <c r="A31" s="2">
+        <v>43160</v>
       </c>
       <c r="E31">
         <v>135</v>
@@ -2837,8 +2844,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32">
-        <v>17622</v>
+      <c r="A32" s="2">
+        <v>43191</v>
       </c>
       <c r="E32">
         <v>125</v>
@@ -2915,8 +2922,8 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33">
-        <v>17652</v>
+      <c r="A33" s="2">
+        <v>43221</v>
       </c>
       <c r="E33">
         <v>141</v>
@@ -2993,8 +3000,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34">
-        <v>17683</v>
+      <c r="A34" s="2">
+        <v>43252</v>
       </c>
       <c r="E34">
         <v>143</v>
@@ -3071,8 +3078,8 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35">
-        <v>17713</v>
+      <c r="A35" s="2">
+        <v>43282</v>
       </c>
       <c r="E35">
         <v>117</v>
@@ -3149,8 +3156,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36">
-        <v>17744</v>
+      <c r="A36" s="2">
+        <v>43313</v>
       </c>
       <c r="E36">
         <v>129</v>
@@ -3227,8 +3234,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37">
-        <v>17775</v>
+      <c r="A37" s="2">
+        <v>43344</v>
       </c>
       <c r="E37">
         <v>114</v>
@@ -3308,8 +3315,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38">
-        <v>17805</v>
+      <c r="A38" s="2">
+        <v>43374</v>
       </c>
       <c r="E38">
         <v>136</v>
@@ -3389,8 +3396,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39">
-        <v>17836</v>
+      <c r="A39" s="2">
+        <v>43405</v>
       </c>
       <c r="B39">
         <v>43</v>
@@ -3479,8 +3486,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40">
-        <v>17866</v>
+      <c r="A40" s="2">
+        <v>43435</v>
       </c>
       <c r="E40">
         <v>127</v>
@@ -3560,8 +3567,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41">
-        <v>17897</v>
+      <c r="A41" s="2">
+        <v>43466</v>
       </c>
       <c r="B41">
         <v>59</v>
@@ -3650,8 +3657,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42">
-        <v>17928</v>
+      <c r="A42" s="2">
+        <v>43497</v>
       </c>
       <c r="E42">
         <v>136</v>
@@ -3731,8 +3738,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43">
-        <v>17956</v>
+      <c r="A43" s="2">
+        <v>43525</v>
       </c>
       <c r="B43">
         <v>69</v>
@@ -3821,8 +3828,8 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44">
-        <v>17987</v>
+      <c r="A44" s="2">
+        <v>43556</v>
       </c>
       <c r="E44">
         <v>115</v>
@@ -3902,8 +3909,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45">
-        <v>18017</v>
+      <c r="A45" s="2">
+        <v>43586</v>
       </c>
       <c r="B45">
         <v>82</v>
@@ -3992,8 +3999,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46">
-        <v>18048</v>
+      <c r="A46" s="2">
+        <v>43617</v>
       </c>
       <c r="E46">
         <v>126</v>
@@ -4073,8 +4080,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47">
-        <v>18078</v>
+      <c r="A47" s="2">
+        <v>43647</v>
       </c>
       <c r="B47">
         <v>105</v>
@@ -4163,8 +4170,8 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48">
-        <v>18109</v>
+      <c r="A48" s="2">
+        <v>43678</v>
       </c>
       <c r="E48">
         <v>124</v>
@@ -4244,8 +4251,8 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49">
-        <v>18140</v>
+      <c r="A49" s="2">
+        <v>43709</v>
       </c>
       <c r="B49">
         <v>64</v>
@@ -4334,8 +4341,8 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50">
-        <v>18170</v>
+      <c r="A50" s="2">
+        <v>43739</v>
       </c>
       <c r="E50">
         <v>136</v>
@@ -4415,8 +4422,8 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51">
-        <v>18201</v>
+      <c r="A51" s="2">
+        <v>43770</v>
       </c>
       <c r="B51">
         <v>64</v>
@@ -4505,8 +4512,8 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52">
-        <v>18231</v>
+      <c r="A52" s="2">
+        <v>43800</v>
       </c>
       <c r="E52">
         <v>150</v>
@@ -4586,8 +4593,8 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53">
-        <v>18262</v>
+      <c r="A53" s="2">
+        <v>43831</v>
       </c>
       <c r="B53">
         <v>46</v>
@@ -4676,8 +4683,8 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54">
-        <v>18293</v>
+      <c r="A54" s="2">
+        <v>43862</v>
       </c>
       <c r="E54">
         <v>168</v>
@@ -4757,8 +4764,8 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55">
-        <v>18322</v>
+      <c r="A55" s="2">
+        <v>43891</v>
       </c>
       <c r="B55">
         <v>48</v>
@@ -4847,8 +4854,8 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56">
-        <v>18353</v>
+      <c r="A56" s="2">
+        <v>43922</v>
       </c>
       <c r="E56">
         <v>96</v>
@@ -4928,8 +4935,8 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57">
-        <v>18383</v>
+      <c r="A57" s="2">
+        <v>43952</v>
       </c>
       <c r="B57">
         <v>51</v>
@@ -5018,8 +5025,8 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58">
-        <v>18414</v>
+      <c r="A58" s="2">
+        <v>43983</v>
       </c>
       <c r="E58">
         <v>117</v>
@@ -5099,8 +5106,8 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59">
-        <v>18444</v>
+      <c r="A59" s="2">
+        <v>44013</v>
       </c>
       <c r="B59">
         <v>52</v>
@@ -5189,8 +5196,8 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60">
-        <v>18475</v>
+      <c r="A60" s="2">
+        <v>44044</v>
       </c>
       <c r="E60">
         <v>144</v>
@@ -5270,8 +5277,8 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61">
-        <v>18506</v>
+      <c r="A61" s="2">
+        <v>44075</v>
       </c>
       <c r="B61">
         <v>74</v>
@@ -5360,8 +5367,8 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62">
-        <v>18536</v>
+      <c r="A62" s="2">
+        <v>44105</v>
       </c>
       <c r="E62">
         <v>183</v>
@@ -5441,8 +5448,8 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63">
-        <v>18567</v>
+      <c r="A63" s="2">
+        <v>44136</v>
       </c>
       <c r="B63">
         <v>76</v>
@@ -5531,8 +5538,8 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64">
-        <v>18597</v>
+      <c r="A64" s="2">
+        <v>44166</v>
       </c>
       <c r="E64">
         <v>174</v>
@@ -5612,8 +5619,8 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65">
-        <v>18628</v>
+      <c r="A65" s="2">
+        <v>44197</v>
       </c>
       <c r="B65">
         <v>78</v>
@@ -5702,8 +5709,8 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66">
-        <v>18659</v>
+      <c r="A66" s="2">
+        <v>44228</v>
       </c>
       <c r="E66">
         <v>165</v>
@@ -5783,8 +5790,8 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67">
-        <v>18687</v>
+      <c r="A67" s="2">
+        <v>44256</v>
       </c>
       <c r="B67">
         <v>88</v>
@@ -5873,8 +5880,8 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68">
-        <v>18718</v>
+      <c r="A68" s="2">
+        <v>44287</v>
       </c>
       <c r="E68">
         <v>178</v>
@@ -5954,8 +5961,8 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69">
-        <v>18748</v>
+      <c r="A69" s="2">
+        <v>44317</v>
       </c>
       <c r="B69">
         <v>87</v>
@@ -6044,8 +6051,8 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70">
-        <v>18779</v>
+      <c r="A70" s="2">
+        <v>44348</v>
       </c>
       <c r="E70">
         <v>137</v>
@@ -6125,8 +6132,8 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71">
-        <v>18809</v>
+      <c r="A71" s="2">
+        <v>44378</v>
       </c>
       <c r="B71">
         <v>74</v>
@@ -6215,8 +6222,8 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72">
-        <v>18840</v>
+      <c r="A72" s="2">
+        <v>44409</v>
       </c>
       <c r="E72">
         <v>138</v>
@@ -6296,8 +6303,8 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73">
-        <v>18871</v>
+      <c r="A73" s="2">
+        <v>44440</v>
       </c>
       <c r="B73">
         <v>79</v>
@@ -6386,8 +6393,8 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74">
-        <v>18901</v>
+      <c r="A74" s="2">
+        <v>44470</v>
       </c>
       <c r="E74">
         <v>121</v>
@@ -6467,8 +6474,8 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75">
-        <v>18932</v>
+      <c r="A75" s="2">
+        <v>44501</v>
       </c>
       <c r="B75">
         <v>75</v>
@@ -6557,8 +6564,8 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76">
-        <v>18962</v>
+      <c r="A76" s="2">
+        <v>44531</v>
       </c>
       <c r="E76">
         <v>125</v>
@@ -6638,8 +6645,8 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77">
-        <v>18993</v>
+      <c r="A77" s="2">
+        <v>44562</v>
       </c>
       <c r="B77">
         <v>94</v>
@@ -6728,8 +6735,8 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78">
-        <v>19024</v>
+      <c r="A78" s="2">
+        <v>44593</v>
       </c>
       <c r="E78">
         <v>125</v>
@@ -6809,8 +6816,8 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79">
-        <v>19052</v>
+      <c r="A79" s="2">
+        <v>44621</v>
       </c>
       <c r="B79">
         <v>87</v>
@@ -6899,8 +6906,8 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80">
-        <v>19083</v>
+      <c r="A80" s="2">
+        <v>44652</v>
       </c>
       <c r="E80">
         <v>121</v>
@@ -6980,8 +6987,8 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81">
-        <v>19113</v>
+      <c r="A81" s="2">
+        <v>44682</v>
       </c>
       <c r="B81">
         <v>97</v>
@@ -7070,8 +7077,8 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82">
-        <v>19144</v>
+      <c r="A82" s="2">
+        <v>44713</v>
       </c>
       <c r="E82">
         <v>97</v>
@@ -7151,8 +7158,8 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83">
-        <v>19174</v>
+      <c r="A83" s="2">
+        <v>44743</v>
       </c>
       <c r="B83">
         <v>70</v>
@@ -7241,8 +7248,8 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84">
-        <v>19205</v>
+      <c r="A84" s="2">
+        <v>44774</v>
       </c>
       <c r="E84">
         <v>117</v>
@@ -7322,8 +7329,8 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85">
-        <v>19236</v>
+      <c r="A85" s="2">
+        <v>44805</v>
       </c>
       <c r="B85">
         <v>71</v>
@@ -7412,8 +7419,8 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86">
-        <v>19266</v>
+      <c r="A86" s="2">
+        <v>44835</v>
       </c>
       <c r="E86">
         <v>102</v>
@@ -7493,8 +7500,8 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87">
-        <v>19297</v>
+      <c r="A87" s="2">
+        <v>44866</v>
       </c>
       <c r="B87">
         <v>45</v>
@@ -7583,8 +7590,8 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88">
-        <v>19327</v>
+      <c r="A88" s="2">
+        <v>44896</v>
       </c>
       <c r="E88">
         <v>126</v>
@@ -7664,8 +7671,8 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89">
-        <v>19358</v>
+      <c r="A89" s="2">
+        <v>44927</v>
       </c>
       <c r="B89">
         <v>38</v>
@@ -7754,8 +7761,8 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90">
-        <v>19389</v>
+      <c r="A90" s="2">
+        <v>44958</v>
       </c>
       <c r="E90">
         <v>125</v>
@@ -7835,8 +7842,8 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91">
-        <v>19417</v>
+      <c r="A91" s="2">
+        <v>44986</v>
       </c>
       <c r="B91">
         <v>35</v>
@@ -7925,8 +7932,8 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92">
-        <v>19448</v>
+      <c r="A92" s="2">
+        <v>45017</v>
       </c>
       <c r="E92">
         <v>123</v>
@@ -8006,8 +8013,8 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93">
-        <v>19478</v>
+      <c r="A93" s="2">
+        <v>45047</v>
       </c>
       <c r="B93">
         <v>31</v>
@@ -8096,8 +8103,8 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94">
-        <v>19509</v>
+      <c r="A94" s="2">
+        <v>45078</v>
       </c>
       <c r="E94">
         <v>121</v>
@@ -8177,8 +8184,8 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95">
-        <v>19539</v>
+      <c r="A95" s="2">
+        <v>45108</v>
       </c>
       <c r="B95">
         <v>35</v>
@@ -8267,8 +8274,8 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96">
-        <v>19570</v>
+      <c r="A96" s="2">
+        <v>45139</v>
       </c>
       <c r="E96">
         <v>115</v>
@@ -8348,8 +8355,8 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97">
-        <v>19601</v>
+      <c r="A97" s="2">
+        <v>45170</v>
       </c>
       <c r="B97">
         <v>39</v>
@@ -8438,8 +8445,8 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98">
-        <v>19631</v>
+      <c r="A98" s="2">
+        <v>45200</v>
       </c>
       <c r="E98">
         <v>110</v>
@@ -8519,8 +8526,8 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99">
-        <v>19662</v>
+      <c r="A99" s="2">
+        <v>45231</v>
       </c>
       <c r="B99">
         <v>47</v>
@@ -8609,8 +8616,8 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100">
-        <v>19692</v>
+      <c r="A100" s="2">
+        <v>45261</v>
       </c>
       <c r="E100">
         <v>114</v>
@@ -8690,8 +8697,8 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101">
-        <v>19723</v>
+      <c r="A101" s="2">
+        <v>45292</v>
       </c>
       <c r="B101">
         <v>68</v>
@@ -8780,8 +8787,8 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102">
-        <v>19754</v>
+      <c r="A102" s="2">
+        <v>45323</v>
       </c>
       <c r="E102">
         <v>111</v>
@@ -8861,8 +8868,8 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103">
-        <v>19783</v>
+      <c r="A103" s="2">
+        <v>45352</v>
       </c>
       <c r="B103">
         <v>79</v>
@@ -8951,8 +8958,8 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104">
-        <v>19814</v>
+      <c r="A104" s="2">
+        <v>45383</v>
       </c>
       <c r="E104">
         <v>99</v>
@@ -9032,8 +9039,8 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105">
-        <v>19844</v>
+      <c r="A105" s="2">
+        <v>45413</v>
       </c>
       <c r="B105">
         <v>90</v>
@@ -9122,8 +9129,8 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106">
-        <v>19875</v>
+      <c r="A106" s="2">
+        <v>45444</v>
       </c>
       <c r="E106">
         <v>105</v>
@@ -9203,8 +9210,8 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107">
-        <v>19905</v>
+      <c r="A107" s="2">
+        <v>45474</v>
       </c>
       <c r="B107">
         <v>106</v>
@@ -9293,8 +9300,8 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108">
-        <v>19936</v>
+      <c r="A108" s="2">
+        <v>45505</v>
       </c>
       <c r="E108">
         <v>100</v>
@@ -9374,8 +9381,8 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109">
-        <v>19967</v>
+      <c r="A109" s="2">
+        <v>45536</v>
       </c>
       <c r="B109">
         <v>105</v>
@@ -9464,8 +9471,8 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110">
-        <v>19997</v>
+      <c r="A110" s="2">
+        <v>45566</v>
       </c>
       <c r="E110">
         <v>115</v>
@@ -9545,8 +9552,8 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111">
-        <v>20028</v>
+      <c r="A111" s="2">
+        <v>45597</v>
       </c>
       <c r="B111">
         <v>120</v>
@@ -9635,8 +9642,8 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112">
-        <v>20058</v>
+      <c r="A112" s="2">
+        <v>45627</v>
       </c>
       <c r="E112">
         <v>136</v>
@@ -9716,8 +9723,8 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113">
-        <v>20089</v>
+      <c r="A113" s="2">
+        <v>45658</v>
       </c>
       <c r="B113">
         <v>81</v>
@@ -9806,8 +9813,8 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114">
-        <v>20120</v>
+      <c r="A114" s="2">
+        <v>45689</v>
       </c>
       <c r="E114">
         <v>152</v>
@@ -9887,8 +9894,8 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115">
-        <v>20148</v>
+      <c r="A115" s="2">
+        <v>45717</v>
       </c>
       <c r="B115">
         <v>100</v>
@@ -9977,8 +9984,8 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116">
-        <v>20179</v>
+      <c r="A116" s="2">
+        <v>45748</v>
       </c>
       <c r="E116">
         <v>148</v>
@@ -10058,8 +10065,8 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117">
-        <v>20209</v>
+      <c r="A117" s="2">
+        <v>45778</v>
       </c>
       <c r="B117">
         <v>94</v>
@@ -10148,8 +10155,8 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118">
-        <v>20240</v>
+      <c r="A118" s="2">
+        <v>45809</v>
       </c>
       <c r="E118">
         <v>146</v>
@@ -10229,8 +10236,8 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119">
-        <v>20270</v>
+      <c r="A119" s="2">
+        <v>45839</v>
       </c>
       <c r="B119">
         <v>89</v>
@@ -10319,8 +10326,8 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120">
-        <v>20301</v>
+      <c r="A120" s="2">
+        <v>45870</v>
       </c>
       <c r="E120">
         <v>125</v>
@@ -10400,8 +10407,8 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121">
-        <v>20332</v>
+      <c r="A121" s="2">
+        <v>45901</v>
       </c>
       <c r="B121">
         <v>87</v>
@@ -10490,8 +10497,8 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122">
-        <v>20362</v>
+      <c r="A122" s="2">
+        <v>45931</v>
       </c>
       <c r="E122">
         <v>129</v>
@@ -10571,8 +10578,8 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123">
-        <v>20393</v>
+      <c r="A123" s="2">
+        <v>45962</v>
       </c>
       <c r="B123">
         <v>124</v>
@@ -10661,8 +10668,8 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124">
-        <v>20423</v>
+      <c r="A124" s="2">
+        <v>45992</v>
       </c>
       <c r="E124">
         <v>136</v>
@@ -10742,8 +10749,8 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125">
-        <v>20454</v>
+      <c r="A125" s="2">
+        <v>46023</v>
       </c>
       <c r="B125">
         <v>132</v>
@@ -10832,8 +10839,8 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126">
-        <v>20485</v>
+      <c r="A126" s="2">
+        <v>46054</v>
       </c>
       <c r="E126">
         <v>116</v>
@@ -10913,8 +10920,8 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127">
-        <v>20513</v>
+      <c r="A127" s="2">
+        <v>46082</v>
       </c>
       <c r="E127">
         <v>127</v>

</xml_diff>